<commit_message>
regular backup (Tue May 27 12:50:02 PM JST 2025)
</commit_message>
<xml_diff>
--- a/xlsx/20250527.xlsx
+++ b/xlsx/20250527.xlsx
@@ -31505,10 +31505,8 @@
           <t>news-20231208-02.html</t>
         </is>
       </c>
-      <c r="D337" t="inlineStr">
-        <is>
-          <t>00000655</t>
-        </is>
+      <c r="D337" t="n">
+        <v>655</v>
       </c>
     </row>
     <row r="338">
@@ -31527,10 +31525,8 @@
           <t>news-20231214-03.html</t>
         </is>
       </c>
-      <c r="D338" t="inlineStr">
-        <is>
-          <t>00000231</t>
-        </is>
+      <c r="D338" t="n">
+        <v>231</v>
       </c>
     </row>
     <row r="339">
@@ -31549,10 +31545,8 @@
           <t>news-20231222-01.html</t>
         </is>
       </c>
-      <c r="D339" t="inlineStr">
-        <is>
-          <t>00000055</t>
-        </is>
+      <c r="D339" t="n">
+        <v>55</v>
       </c>
     </row>
     <row r="340">
@@ -31571,10 +31565,8 @@
           <t>news-20240105-01.html</t>
         </is>
       </c>
-      <c r="D340" t="inlineStr">
-        <is>
-          <t>00000074</t>
-        </is>
+      <c r="D340" t="n">
+        <v>74</v>
       </c>
     </row>
     <row r="341">
@@ -31593,10 +31585,8 @@
           <t>news-20240112-05.html</t>
         </is>
       </c>
-      <c r="D341" t="inlineStr">
-        <is>
-          <t>00000028</t>
-        </is>
+      <c r="D341" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="342">
@@ -31615,10 +31605,8 @@
           <t>news-20240119-03.html</t>
         </is>
       </c>
-      <c r="D342" t="inlineStr">
-        <is>
-          <t>00000024</t>
-        </is>
+      <c r="D342" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="343">
@@ -31637,10 +31625,8 @@
           <t>news-20240126-02.html</t>
         </is>
       </c>
-      <c r="D343" t="inlineStr">
-        <is>
-          <t>00000028</t>
-        </is>
+      <c r="D343" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="344">
@@ -31659,10 +31645,8 @@
           <t>news-20240202-03.html</t>
         </is>
       </c>
-      <c r="D344" t="inlineStr">
-        <is>
-          <t>00000017</t>
-        </is>
+      <c r="D344" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="345">
@@ -31681,10 +31665,8 @@
           <t>news-20240209-03.html</t>
         </is>
       </c>
-      <c r="D345" t="inlineStr">
-        <is>
-          <t>00000012</t>
-        </is>
+      <c r="D345" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="346">
@@ -31703,10 +31685,8 @@
           <t>news-20240216-03.html</t>
         </is>
       </c>
-      <c r="D346" t="inlineStr">
-        <is>
-          <t>00000008</t>
-        </is>
+      <c r="D346" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="347">
@@ -31725,10 +31705,8 @@
           <t>news-20240301-03.html</t>
         </is>
       </c>
-      <c r="D347" t="inlineStr">
-        <is>
-          <t>00000022</t>
-        </is>
+      <c r="D347" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="348">
@@ -31747,10 +31725,8 @@
           <t>news-20240307-02.html</t>
         </is>
       </c>
-      <c r="D348" t="inlineStr">
-        <is>
-          <t>00000018</t>
-        </is>
+      <c r="D348" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="349">
@@ -31769,10 +31745,8 @@
           <t>news-20240315-04.html</t>
         </is>
       </c>
-      <c r="D349" t="inlineStr">
-        <is>
-          <t>00000020</t>
-        </is>
+      <c r="D349" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="350">
@@ -31791,10 +31765,8 @@
           <t>news-20240322-01.html</t>
         </is>
       </c>
-      <c r="D350" t="inlineStr">
-        <is>
-          <t>00000026</t>
-        </is>
+      <c r="D350" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="351">
@@ -31813,10 +31785,8 @@
           <t>news-20240329-05.html</t>
         </is>
       </c>
-      <c r="D351" t="inlineStr">
-        <is>
-          <t>00000130</t>
-        </is>
+      <c r="D351" t="n">
+        <v>130</v>
       </c>
     </row>
     <row r="352">
@@ -31835,10 +31805,8 @@
           <t>news-20240405-03.html</t>
         </is>
       </c>
-      <c r="D352" t="inlineStr">
-        <is>
-          <t>00000017</t>
-        </is>
+      <c r="D352" t="n">
+        <v>17</v>
       </c>
     </row>
     <row r="353">
@@ -31857,10 +31825,8 @@
           <t>news-20240412-07.html</t>
         </is>
       </c>
-      <c r="D353" t="inlineStr">
-        <is>
-          <t>00000025</t>
-        </is>
+      <c r="D353" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="354">
@@ -31879,10 +31845,8 @@
           <t>news-20240419-03.html</t>
         </is>
       </c>
-      <c r="D354" t="inlineStr">
-        <is>
-          <t>00017504</t>
-        </is>
+      <c r="D354" t="n">
+        <v>17504</v>
       </c>
     </row>
     <row r="355">
@@ -31901,10 +31865,8 @@
           <t>news-20240426-07.html</t>
         </is>
       </c>
-      <c r="D355" t="inlineStr">
-        <is>
-          <t>00000021</t>
-        </is>
+      <c r="D355" t="n">
+        <v>21</v>
       </c>
     </row>
     <row r="356">
@@ -31923,10 +31885,8 @@
           <t>news-20240510-01.html</t>
         </is>
       </c>
-      <c r="D356" t="inlineStr">
-        <is>
-          <t>00000092</t>
-        </is>
+      <c r="D356" t="n">
+        <v>92</v>
       </c>
     </row>
     <row r="357">
@@ -31945,10 +31905,8 @@
           <t>news-20240517-01.html</t>
         </is>
       </c>
-      <c r="D357" t="inlineStr">
-        <is>
-          <t>00000020</t>
-        </is>
+      <c r="D357" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="358">
@@ -31967,10 +31925,8 @@
           <t>news-20240524-01.html</t>
         </is>
       </c>
-      <c r="D358" t="inlineStr">
-        <is>
-          <t>00000039</t>
-        </is>
+      <c r="D358" t="n">
+        <v>39</v>
       </c>
     </row>
     <row r="359">
@@ -31989,10 +31945,8 @@
           <t>news-20240531-02.html</t>
         </is>
       </c>
-      <c r="D359" t="inlineStr">
-        <is>
-          <t>00000043</t>
-        </is>
+      <c r="D359" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="360">
@@ -32011,10 +31965,8 @@
           <t>news-20240607-01.html</t>
         </is>
       </c>
-      <c r="D360" t="inlineStr">
-        <is>
-          <t>00000023</t>
-        </is>
+      <c r="D360" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="361">
@@ -32033,10 +31985,8 @@
           <t>news-20240614-03.html</t>
         </is>
       </c>
-      <c r="D361" t="inlineStr">
-        <is>
-          <t>00000025</t>
-        </is>
+      <c r="D361" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="362">
@@ -32055,10 +32005,8 @@
           <t>news-20240621-02.html</t>
         </is>
       </c>
-      <c r="D362" t="inlineStr">
-        <is>
-          <t>00000047</t>
-        </is>
+      <c r="D362" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="363">
@@ -32077,10 +32025,8 @@
           <t>news-20240628-03.html</t>
         </is>
       </c>
-      <c r="D363" t="inlineStr">
-        <is>
-          <t>00001118</t>
-        </is>
+      <c r="D363" t="n">
+        <v>1118</v>
       </c>
     </row>
     <row r="364">
@@ -32099,10 +32045,8 @@
           <t>news-20240705-01.html</t>
         </is>
       </c>
-      <c r="D364" t="inlineStr">
-        <is>
-          <t>00000032</t>
-        </is>
+      <c r="D364" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="365">
@@ -32121,10 +32065,8 @@
           <t>news-20240712-03.html</t>
         </is>
       </c>
-      <c r="D365" t="inlineStr">
-        <is>
-          <t>00000014</t>
-        </is>
+      <c r="D365" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="366">
@@ -32143,10 +32085,8 @@
           <t>news-20240719-10.html</t>
         </is>
       </c>
-      <c r="D366" t="inlineStr">
-        <is>
-          <t>00000025</t>
-        </is>
+      <c r="D366" t="n">
+        <v>25</v>
       </c>
     </row>
     <row r="367">
@@ -32165,10 +32105,8 @@
           <t>news-20240726-02.html</t>
         </is>
       </c>
-      <c r="D367" t="inlineStr">
-        <is>
-          <t>00000031</t>
-        </is>
+      <c r="D367" t="n">
+        <v>31</v>
       </c>
     </row>
     <row r="368">
@@ -32187,10 +32125,8 @@
           <t>news-20240802-02.html</t>
         </is>
       </c>
-      <c r="D368" t="inlineStr">
-        <is>
-          <t>00000028</t>
-        </is>
+      <c r="D368" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="369">
@@ -32209,10 +32145,8 @@
           <t>news-20240809-01.html</t>
         </is>
       </c>
-      <c r="D369" t="inlineStr">
-        <is>
-          <t>00000033</t>
-        </is>
+      <c r="D369" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="370">
@@ -32231,10 +32165,8 @@
           <t>news-20240816-01.html</t>
         </is>
       </c>
-      <c r="D370" t="inlineStr">
-        <is>
-          <t>00000033</t>
-        </is>
+      <c r="D370" t="n">
+        <v>33</v>
       </c>
     </row>
     <row r="371">
@@ -32253,10 +32185,8 @@
           <t>news-20240823-03.html</t>
         </is>
       </c>
-      <c r="D371" t="inlineStr">
-        <is>
-          <t>00000032</t>
-        </is>
+      <c r="D371" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="372">
@@ -32275,10 +32205,8 @@
           <t>news-20240830-06.html</t>
         </is>
       </c>
-      <c r="D372" t="inlineStr">
-        <is>
-          <t>00000062</t>
-        </is>
+      <c r="D372" t="n">
+        <v>62</v>
       </c>
     </row>
     <row r="373">
@@ -32297,10 +32225,8 @@
           <t>news-20240906-04.html</t>
         </is>
       </c>
-      <c r="D373" t="inlineStr">
-        <is>
-          <t>00000068</t>
-        </is>
+      <c r="D373" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="374">
@@ -32319,10 +32245,8 @@
           <t>news-20240913-03.html</t>
         </is>
       </c>
-      <c r="D374" t="inlineStr">
-        <is>
-          <t>00000076</t>
-        </is>
+      <c r="D374" t="n">
+        <v>76</v>
       </c>
     </row>
     <row r="375">
@@ -32341,10 +32265,8 @@
           <t>news-20240920-04.html</t>
         </is>
       </c>
-      <c r="D375" t="inlineStr">
-        <is>
-          <t>00000079</t>
-        </is>
+      <c r="D375" t="n">
+        <v>79</v>
       </c>
     </row>
     <row r="376">
@@ -32363,10 +32285,8 @@
           <t>news-20240927-02.html</t>
         </is>
       </c>
-      <c r="D376" t="inlineStr">
-        <is>
-          <t>00000175</t>
-        </is>
+      <c r="D376" t="n">
+        <v>175</v>
       </c>
     </row>
     <row r="377">
@@ -32385,10 +32305,8 @@
           <t>news-20241004-07.html</t>
         </is>
       </c>
-      <c r="D377" t="inlineStr">
-        <is>
-          <t>00000322</t>
-        </is>
+      <c r="D377" t="n">
+        <v>322</v>
       </c>
     </row>
     <row r="378">
@@ -32407,10 +32325,8 @@
           <t>news-20241011-05.html</t>
         </is>
       </c>
-      <c r="D378" t="inlineStr">
-        <is>
-          <t>00001891</t>
-        </is>
+      <c r="D378" t="n">
+        <v>1891</v>
       </c>
     </row>
     <row r="379">
@@ -32429,10 +32345,8 @@
           <t>news-20241018-01.html</t>
         </is>
       </c>
-      <c r="D379" t="inlineStr">
-        <is>
-          <t>00000122</t>
-        </is>
+      <c r="D379" t="n">
+        <v>122</v>
       </c>
     </row>
     <row r="380">
@@ -32451,10 +32365,8 @@
           <t>news-20241025-04.html</t>
         </is>
       </c>
-      <c r="D380" t="inlineStr">
-        <is>
-          <t>00000063</t>
-        </is>
+      <c r="D380" t="n">
+        <v>63</v>
       </c>
     </row>
     <row r="381">
@@ -32473,10 +32385,8 @@
           <t>news-20241101-01.html</t>
         </is>
       </c>
-      <c r="D381" t="inlineStr">
-        <is>
-          <t>00000067</t>
-        </is>
+      <c r="D381" t="n">
+        <v>67</v>
       </c>
     </row>
     <row r="382">
@@ -32495,10 +32405,8 @@
           <t>news-20241108-03.html</t>
         </is>
       </c>
-      <c r="D382" t="inlineStr">
-        <is>
-          <t>00000068</t>
-        </is>
+      <c r="D382" t="n">
+        <v>68</v>
       </c>
     </row>
     <row r="383">
@@ -32517,10 +32425,8 @@
           <t>news-20241115-03.html</t>
         </is>
       </c>
-      <c r="D383" t="inlineStr">
-        <is>
-          <t>00000050</t>
-        </is>
+      <c r="D383" t="n">
+        <v>50</v>
       </c>
     </row>
     <row r="384">
@@ -32539,10 +32445,8 @@
           <t>news-20241122-03.html</t>
         </is>
       </c>
-      <c r="D384" t="inlineStr">
-        <is>
-          <t>00000057</t>
-        </is>
+      <c r="D384" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="385">
@@ -32561,10 +32465,8 @@
           <t>news-20241129-04.html</t>
         </is>
       </c>
-      <c r="D385" t="inlineStr">
-        <is>
-          <t>00000047</t>
-        </is>
+      <c r="D385" t="n">
+        <v>47</v>
       </c>
     </row>
     <row r="386">
@@ -32583,10 +32485,8 @@
           <t>news-20241206-1.html</t>
         </is>
       </c>
-      <c r="D386" t="inlineStr">
-        <is>
-          <t>00000069</t>
-        </is>
+      <c r="D386" t="n">
+        <v>69</v>
       </c>
     </row>
     <row r="387">
@@ -32605,10 +32505,8 @@
           <t>news-20241213-01.html</t>
         </is>
       </c>
-      <c r="D387" t="inlineStr">
-        <is>
-          <t>00000043</t>
-        </is>
+      <c r="D387" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="388">
@@ -32627,10 +32525,8 @@
           <t>news-20241220-05.html</t>
         </is>
       </c>
-      <c r="D388" t="inlineStr">
-        <is>
-          <t>00000087</t>
-        </is>
+      <c r="D388" t="n">
+        <v>87</v>
       </c>
     </row>
     <row r="389">
@@ -32649,10 +32545,8 @@
           <t>news-20241227-06.html</t>
         </is>
       </c>
-      <c r="D389" t="inlineStr">
-        <is>
-          <t>00000064</t>
-        </is>
+      <c r="D389" t="n">
+        <v>64</v>
       </c>
     </row>
     <row r="390">
@@ -32671,10 +32565,8 @@
           <t>news-20250110-06.html</t>
         </is>
       </c>
-      <c r="D390" t="inlineStr">
-        <is>
-          <t>00000382</t>
-        </is>
+      <c r="D390" t="n">
+        <v>382</v>
       </c>
     </row>
     <row r="391">
@@ -32693,10 +32585,8 @@
           <t>news-20250117-02.html</t>
         </is>
       </c>
-      <c r="D391" t="inlineStr">
-        <is>
-          <t>00000229</t>
-        </is>
+      <c r="D391" t="n">
+        <v>229</v>
       </c>
     </row>
     <row r="392">
@@ -32715,10 +32605,8 @@
           <t>news-20250124-02.html</t>
         </is>
       </c>
-      <c r="D392" t="inlineStr">
-        <is>
-          <t>00000227</t>
-        </is>
+      <c r="D392" t="n">
+        <v>227</v>
       </c>
     </row>
     <row r="393">
@@ -32737,10 +32625,8 @@
           <t>news-20250131-01.html</t>
         </is>
       </c>
-      <c r="D393" t="inlineStr">
-        <is>
-          <t>00000245</t>
-        </is>
+      <c r="D393" t="n">
+        <v>245</v>
       </c>
     </row>
     <row r="394">
@@ -32759,10 +32645,8 @@
           <t>news-20250207-03-2.html</t>
         </is>
       </c>
-      <c r="D394" t="inlineStr">
-        <is>
-          <t>00000244</t>
-        </is>
+      <c r="D394" t="n">
+        <v>244</v>
       </c>
     </row>
     <row r="395">
@@ -32781,10 +32665,8 @@
           <t>news-20250214-05.html</t>
         </is>
       </c>
-      <c r="D395" t="inlineStr">
-        <is>
-          <t>00000308</t>
-        </is>
+      <c r="D395" t="n">
+        <v>308</v>
       </c>
     </row>
     <row r="396">
@@ -32803,10 +32685,8 @@
           <t>news-20250221-05.html</t>
         </is>
       </c>
-      <c r="D396" t="inlineStr">
-        <is>
-          <t>00000275</t>
-        </is>
+      <c r="D396" t="n">
+        <v>275</v>
       </c>
     </row>
     <row r="397">
@@ -32825,10 +32705,8 @@
           <t>news-20250228-02.html</t>
         </is>
       </c>
-      <c r="D397" t="inlineStr">
-        <is>
-          <t>00000304</t>
-        </is>
+      <c r="D397" t="n">
+        <v>304</v>
       </c>
     </row>
     <row r="398">
@@ -32847,10 +32725,8 @@
           <t>news-20250307-03.html</t>
         </is>
       </c>
-      <c r="D398" t="inlineStr">
-        <is>
-          <t>00000395</t>
-        </is>
+      <c r="D398" t="n">
+        <v>395</v>
       </c>
     </row>
     <row r="399">
@@ -32869,10 +32745,8 @@
           <t>news-20250314-01-02.html</t>
         </is>
       </c>
-      <c r="D399" t="inlineStr">
-        <is>
-          <t>00000462</t>
-        </is>
+      <c r="D399" t="n">
+        <v>462</v>
       </c>
     </row>
     <row r="400">
@@ -32891,10 +32765,8 @@
           <t>news-20250321-04.html</t>
         </is>
       </c>
-      <c r="D400" t="inlineStr">
-        <is>
-          <t>00000549</t>
-        </is>
+      <c r="D400" t="n">
+        <v>549</v>
       </c>
     </row>
     <row r="401">
@@ -32913,10 +32785,8 @@
           <t>news-20250328-01.html</t>
         </is>
       </c>
-      <c r="D401" t="inlineStr">
-        <is>
-          <t>00000618</t>
-        </is>
+      <c r="D401" t="n">
+        <v>618</v>
       </c>
     </row>
     <row r="402">
@@ -32935,10 +32805,8 @@
           <t>news-20250404-02.html</t>
         </is>
       </c>
-      <c r="D402" t="inlineStr">
-        <is>
-          <t>00000935</t>
-        </is>
+      <c r="D402" t="n">
+        <v>935</v>
       </c>
     </row>
     <row r="403">
@@ -32957,10 +32825,8 @@
           <t>news-20250411-03.html</t>
         </is>
       </c>
-      <c r="D403" t="inlineStr">
-        <is>
-          <t>00001713</t>
-        </is>
+      <c r="D403" t="n">
+        <v>1713</v>
       </c>
     </row>
     <row r="404">
@@ -44299,10 +44165,8 @@
           <t>news-20250421-02.html</t>
         </is>
       </c>
-      <c r="D970" t="inlineStr">
-        <is>
-          <t>00006334</t>
-        </is>
+      <c r="D970" t="n">
+        <v>6334</v>
       </c>
     </row>
     <row r="971">
@@ -44321,10 +44185,8 @@
           <t>news-20250428-01.html</t>
         </is>
       </c>
-      <c r="D971" t="inlineStr">
-        <is>
-          <t>00003011</t>
-        </is>
+      <c r="D971" t="n">
+        <v>3011</v>
       </c>
     </row>
     <row r="972">
@@ -44343,10 +44205,8 @@
           <t>news-20250505-02.html</t>
         </is>
       </c>
-      <c r="D972" t="inlineStr">
-        <is>
-          <t>00003908</t>
-        </is>
+      <c r="D972" t="n">
+        <v>3908</v>
       </c>
     </row>
     <row r="973">
@@ -44365,10 +44225,8 @@
           <t>news-20250512-02.html</t>
         </is>
       </c>
-      <c r="D973" t="inlineStr">
-        <is>
-          <t>00006017</t>
-        </is>
+      <c r="D973" t="n">
+        <v>6017</v>
       </c>
     </row>
     <row r="974">
@@ -44387,10 +44245,8 @@
           <t>news-20250519-01.html</t>
         </is>
       </c>
-      <c r="D974" t="inlineStr">
-        <is>
-          <t>00007251</t>
-        </is>
+      <c r="D974" t="n">
+        <v>7251</v>
       </c>
     </row>
     <row r="975">
@@ -44409,10 +44265,8 @@
           <t>news-20250526-01.html</t>
         </is>
       </c>
-      <c r="D975" t="inlineStr">
-        <is>
-          <t>00010761</t>
-        </is>
+      <c r="D975" t="n">
+        <v>10761</v>
       </c>
     </row>
     <row r="976">

</xml_diff>